<commit_message>
8th Oct 2026 reports
</commit_message>
<xml_diff>
--- a/data/Oct/Data_Oct.xlsx
+++ b/data/Oct/Data_Oct.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Oct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01642EC6-5834-4370-8D55-5950767944B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC6584E-729B-4993-97DD-35D4F5395031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-10" sheetId="6" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="05-10" sheetId="9" r:id="rId4"/>
     <sheet name="06-10" sheetId="10" r:id="rId5"/>
     <sheet name="07-10" sheetId="11" r:id="rId6"/>
+    <sheet name="08-10" sheetId="12" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2525" uniqueCount="878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2738" uniqueCount="939">
   <si>
     <t>THU 5</t>
   </si>
@@ -2380,6 +2381,9 @@
     <t>41A Huỳnh Tịnh của p19</t>
   </si>
   <si>
+    <t>kh ck shop 1340k</t>
+  </si>
+  <si>
     <t>Ngọc Ánh</t>
   </si>
   <si>
@@ -2389,39 +2393,63 @@
     <t>2/21 phan thúc duyện</t>
   </si>
   <si>
+    <t>BN6352</t>
+  </si>
+  <si>
     <t>HD064708</t>
   </si>
   <si>
+    <t>Tú Oanh - fb Không Nói Xâm</t>
+  </si>
+  <si>
+    <t>HD064593</t>
+  </si>
+  <si>
+    <t>69 Dương Đình Nghệ P8</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
     <t>AT 07-10</t>
   </si>
   <si>
-    <t>Tú Oanh - fb Không Nói Xâm</t>
-  </si>
-  <si>
-    <t>HD064593</t>
-  </si>
-  <si>
-    <t>69 Dương Đình Nghệ P8</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
     <t>Đinh Thị Thu Hà</t>
   </si>
   <si>
     <t>HD064612</t>
   </si>
   <si>
+    <t>176/1 Nguyễn Văn Thương, P. Thạnh Mỹ Tây</t>
+  </si>
+  <si>
     <t>HD064640</t>
   </si>
   <si>
+    <t>mỹ huyền</t>
+  </si>
+  <si>
     <t>HD064774</t>
   </si>
   <si>
+    <t>hẻm 2581/27 ấp4 đường huỳnh tấn phát, xã phú xuân</t>
+  </si>
+  <si>
+    <t>kh ck shop 825k</t>
+  </si>
+  <si>
+    <t>Sang - fb Ivy Thụy Pham sale</t>
+  </si>
+  <si>
     <t>HD064668</t>
   </si>
   <si>
+    <t>349/175 Lê Đại Hành Phường Phú Thọ</t>
+  </si>
+  <si>
+    <t>Doan Ngoc Anh Thu</t>
+  </si>
+  <si>
     <t>HD064813</t>
   </si>
   <si>
@@ -2434,6 +2462,9 @@
     <t>HD064748</t>
   </si>
   <si>
+    <t>32/16a đường số 6, P. BHHA</t>
+  </si>
+  <si>
     <t>Thu Ba DS</t>
   </si>
   <si>
@@ -2455,12 +2486,21 @@
     <t>chị Thu Dương</t>
   </si>
   <si>
+    <t>HD064786</t>
+  </si>
+  <si>
+    <t>158 đào duy anh, P. đức nhuận</t>
+  </si>
+  <si>
     <t>Linh Dịu Dàng</t>
   </si>
   <si>
     <t>HD064810</t>
   </si>
   <si>
+    <t>362/22 lê đức thọ an nhơn</t>
+  </si>
+  <si>
     <t>Kelly Phan</t>
   </si>
   <si>
@@ -2476,18 +2516,27 @@
     <t>HD064778</t>
   </si>
   <si>
+    <t>Angelica Lumiere, Vinhome Grand Park, Phường long bình</t>
+  </si>
+  <si>
     <t>Chip Chip</t>
   </si>
   <si>
     <t>HD064771</t>
   </si>
   <si>
+    <t>71/16 thới an 16</t>
+  </si>
+  <si>
     <t>Trần Thu Hường</t>
   </si>
   <si>
     <t>HD064655</t>
   </si>
   <si>
+    <t>124/28 nguyễn văn cừ, p.cầu ông lãnh</t>
+  </si>
+  <si>
     <t>Vũ Hồng Ly</t>
   </si>
   <si>
@@ -2497,6 +2546,9 @@
     <t>240/29, Hiệp Thành 13, P Tân Thới Hiệp</t>
   </si>
   <si>
+    <t>Cin Vo</t>
+  </si>
+  <si>
     <t>HD064606</t>
   </si>
   <si>
@@ -2509,24 +2561,48 @@
     <t>HD064666</t>
   </si>
   <si>
+    <t>Saicon riverside complex (block C1) Số 4 đào trí phú thuận</t>
+  </si>
+  <si>
+    <t>Thu Pham</t>
+  </si>
+  <si>
     <t>HD064657</t>
   </si>
   <si>
+    <t>chung cư Terra Royal 280 nam kỳ khởi nghĩa, phường võ thị sáu</t>
+  </si>
+  <si>
     <t>HD064688</t>
   </si>
   <si>
+    <t>sldraalvinaa_</t>
+  </si>
+  <si>
     <t>HD064502</t>
   </si>
   <si>
+    <t>1 Đường Số 15 Villa 01 David, An Khánh</t>
+  </si>
+  <si>
     <t>My My</t>
   </si>
   <si>
     <t>HD064651</t>
   </si>
   <si>
+    <t>CC TOPAZ ELITE PHOENIX 1A</t>
+  </si>
+  <si>
+    <t>Trang Nguyen</t>
+  </si>
+  <si>
     <t>HD064597</t>
   </si>
   <si>
+    <t>Bệnh viện 1A - lý thường kiệt</t>
+  </si>
+  <si>
     <t>Ngọc Ngân</t>
   </si>
   <si>
@@ -2551,6 +2627,12 @@
     <t>HD064709</t>
   </si>
   <si>
+    <t>813 Trần Xuân Soạn</t>
+  </si>
+  <si>
+    <t>Nghi</t>
+  </si>
+  <si>
     <t>HD064749</t>
   </si>
   <si>
@@ -2566,115 +2648,217 @@
     <t>1041/19/7 Trần Xuân Soạn</t>
   </si>
   <si>
+    <t>kh ck shop 730k</t>
+  </si>
+  <si>
+    <t>Lê Thị Minh Phượng</t>
+  </si>
+  <si>
     <t>HD064664</t>
   </si>
   <si>
+    <t>101/20 đường số 9 phường bình hưng hòa</t>
+  </si>
+  <si>
     <t>Chau Nguyen</t>
   </si>
   <si>
     <t>HD064811</t>
   </si>
   <si>
+    <t>2555 QL1A Phường Tân Hưng Thuận</t>
+  </si>
+  <si>
     <t>MINZZY</t>
   </si>
   <si>
+    <t>XE TOÀN THẮNG VỀ CÀ PHÊ PHONG LONG THÀNH ĐỒNG NAI</t>
+  </si>
+  <si>
+    <t>HOANG ANH</t>
+  </si>
+  <si>
     <t>385/4 quang trung p go vap</t>
   </si>
   <si>
-    <t>XE TOÀN THẮNG VỀ CÀ PHÊ PHONG LONG THÀNH ĐỒNG NAI</t>
-  </si>
-  <si>
-    <t>HOANG ANH</t>
-  </si>
-  <si>
     <t>vi hồ</t>
   </si>
   <si>
     <t>Nhà xe Minh Quốc</t>
   </si>
   <si>
-    <t>Angelica Lumiere, Vinhome Grand Park, Phường long bình</t>
-  </si>
-  <si>
-    <t>176/1 Nguyễn Văn Thương, P. Thạnh Mỹ Tây</t>
-  </si>
-  <si>
-    <t>Doan Ngoc Anh Thu</t>
-  </si>
-  <si>
-    <t>362/22 lê đức thọ an nhơn</t>
-  </si>
-  <si>
-    <t>71/16 thới an 16</t>
-  </si>
-  <si>
-    <t>BN6352</t>
-  </si>
-  <si>
-    <t>sldraalvinaa_</t>
-  </si>
-  <si>
-    <t>1 Đường Số 15 Villa 01 David, An Khánh</t>
-  </si>
-  <si>
-    <t>HD064786</t>
-  </si>
-  <si>
-    <t>158 đào duy anh, P. đức nhuận</t>
-  </si>
-  <si>
-    <t>Thu Pham</t>
-  </si>
-  <si>
-    <t>chung cư Terra Royal 280 nam kỳ khởi nghĩa, phường võ thị sáu</t>
-  </si>
-  <si>
-    <t>Trang Nguyen</t>
-  </si>
-  <si>
-    <t>Bệnh viện 1A - lý thường kiệt</t>
-  </si>
-  <si>
-    <t>124/28 nguyễn văn cừ, p.cầu ông lãnh</t>
-  </si>
-  <si>
-    <t>CC TOPAZ ELITE PHOENIX 1A</t>
-  </si>
-  <si>
-    <t>813 Trần Xuân Soạn</t>
-  </si>
-  <si>
-    <t>Sang - fb Ivy Thụy Pham sale</t>
-  </si>
-  <si>
-    <t>349/175 Lê Đại Hành Phường Phú Thọ</t>
-  </si>
-  <si>
-    <t>Saicon riverside complex (block C1) Số 4 đào trí phú thuận</t>
-  </si>
-  <si>
-    <t>mỹ huyền</t>
-  </si>
-  <si>
-    <t>hẻm 2581/27 ấp4 đường huỳnh tấn phát, xã phú xuân</t>
-  </si>
-  <si>
-    <t>2555 QL1A Phường Tân Hưng Thuận</t>
-  </si>
-  <si>
-    <t>Nghi</t>
-  </si>
-  <si>
-    <t>32/16a đường số 6, P. BHHA</t>
-  </si>
-  <si>
-    <t>Cin Vo</t>
-  </si>
-  <si>
-    <t>Lê Thị Minh Phượng</t>
-  </si>
-  <si>
-    <t>101/20 đường số 9 phường bình hưng hòa</t>
+    <t>NGAY 8-10</t>
+  </si>
+  <si>
+    <t>Lữ Hạnh Hoàng Châu</t>
+  </si>
+  <si>
+    <t>HD064950</t>
+  </si>
+  <si>
+    <t>17 mai chí thọ phường an khánh New city - toa hawai 1</t>
+  </si>
+  <si>
+    <t>08-10-2026</t>
+  </si>
+  <si>
+    <t>HD065026</t>
+  </si>
+  <si>
+    <t>Bonnie Ya</t>
+  </si>
+  <si>
+    <t>HD065049</t>
+  </si>
+  <si>
+    <t>AT 08-10</t>
+  </si>
+  <si>
+    <t>Lin (Zalo)</t>
+  </si>
+  <si>
+    <t>HD064959</t>
+  </si>
+  <si>
+    <t>mimi (giao cho lễ tân báo hàng của Mimi)</t>
+  </si>
+  <si>
+    <t>HD065007</t>
+  </si>
+  <si>
+    <t>Phạm Huỳnh Duyên</t>
+  </si>
+  <si>
+    <t>HD065071</t>
+  </si>
+  <si>
+    <t>Khánh Hòa</t>
+  </si>
+  <si>
+    <t>HD064924</t>
+  </si>
+  <si>
+    <t>Bảy nhận dùm My Trà</t>
+  </si>
+  <si>
+    <t>HD065006</t>
+  </si>
+  <si>
+    <t>HD065035</t>
+  </si>
+  <si>
+    <t>HD064963</t>
+  </si>
+  <si>
+    <t>HD064863</t>
+  </si>
+  <si>
+    <t>76 Cù Lao</t>
+  </si>
+  <si>
+    <t>Linh Phùng</t>
+  </si>
+  <si>
+    <t>HD065046</t>
+  </si>
+  <si>
+    <t>Ngô thị Thu Thủy - fb Minh Minh Ng</t>
+  </si>
+  <si>
+    <t>HD064954</t>
+  </si>
+  <si>
+    <t>HD064899</t>
+  </si>
+  <si>
+    <t>Khánh Vân</t>
+  </si>
+  <si>
+    <t>HD064868</t>
+  </si>
+  <si>
+    <t>77/39 Kinh Dương Vương F12</t>
+  </si>
+  <si>
+    <t>Trang Angels</t>
+  </si>
+  <si>
+    <t>HD064874</t>
+  </si>
+  <si>
+    <t>Hanna Bui</t>
+  </si>
+  <si>
+    <t>HD064941</t>
+  </si>
+  <si>
+    <t>9B duong 16A Pbinh Hưng hòa A</t>
+  </si>
+  <si>
+    <t>TUYẾT NHI ZL2</t>
+  </si>
+  <si>
+    <t>170F Tân Hoà Đông f14</t>
+  </si>
+  <si>
+    <t>208 nguyễn hữu cảnh phường 22 chung cư vinhome tòa lanmark 5</t>
+  </si>
+  <si>
+    <t>số 42/43-45 Nguyễn Minh Hoàng, phường 12</t>
+  </si>
+  <si>
+    <t>439/97/12 tân thới hiệp 21</t>
+  </si>
+  <si>
+    <t>Em Na</t>
+  </si>
+  <si>
+    <t>16/2 THÁI THỊ NHẠN P10</t>
+  </si>
+  <si>
+    <t>Như Ý Nguyễn</t>
+  </si>
+  <si>
+    <t>4 Đào Trí, P. Phú Thuận</t>
+  </si>
+  <si>
+    <t>nhà 20 đường 2B phường Tân mỹ</t>
+  </si>
+  <si>
+    <t>Ship đến saigon royal 9 Đ. Nguyễn Trường Tộ, Xóm Chiếu</t>
+  </si>
+  <si>
+    <t>35 đặng đức thuật, chung cư RIVERPARK PREMIER Block A, P. Tân Hưng</t>
+  </si>
+  <si>
+    <t>Trang Hồ Vĩnh Như</t>
+  </si>
+  <si>
+    <t>9 Đ. Nguyễn Trường Tộ, Xóm Chiếu</t>
+  </si>
+  <si>
+    <t>491/24/22 nguyễn đình chiểu p2</t>
+  </si>
+  <si>
+    <t>32 đường 85 tân hưng</t>
+  </si>
+  <si>
+    <t>339/24B Đ. Lê Văn Sỹ, Phường 13</t>
+  </si>
+  <si>
+    <t>174/50 Lý chính Thắng.Phường Xuân Hòa</t>
+  </si>
+  <si>
+    <t>932A1 Trường Sa, P. Nhiêu Lộc (ngay tiệm cafe giặt sấy Mộc - lên lầu 1 là tới studio)</t>
+  </si>
+  <si>
+    <t>Trang Nguyễn</t>
+  </si>
+  <si>
+    <t>SS3164-Mr.skill) SS Cargo Shipping (cờn dư 715k)</t>
+  </si>
+  <si>
+    <t>674 đường số 2, Phường 13</t>
   </si>
 </sst>
 </file>
@@ -12925,10 +13109,12 @@
   <dimension ref="A1:P39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="59.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.42578125" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -13047,14 +13233,14 @@
         <v>75</v>
       </c>
       <c r="G4" s="3">
-        <v>1340</v>
+        <v>0</v>
       </c>
       <c r="H4" s="3">
         <v>20</v>
       </c>
       <c r="I4" s="3">
         <f t="shared" si="0"/>
-        <v>1320</v>
+        <v>-20</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>24</v>
@@ -13065,19 +13251,22 @@
       <c r="L4" s="3" t="s">
         <v>775</v>
       </c>
+      <c r="M4" s="3" t="s">
+        <v>779</v>
+      </c>
     </row>
     <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>152</v>
@@ -13110,10 +13299,10 @@
         <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>855</v>
+        <v>783</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>78</v>
@@ -13146,16 +13335,16 @@
         <v>19</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="G7" s="7">
         <v>0</v>
@@ -13168,7 +13357,7 @@
         <v>-25</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>24</v>
@@ -13182,13 +13371,13 @@
         <v>19</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>851</v>
+        <v>792</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>75</v>
@@ -13218,13 +13407,13 @@
         <v>19</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>152</v>
@@ -13257,29 +13446,29 @@
         <v>19</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>870</v>
+        <v>794</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>871</v>
+        <v>796</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>199</v>
       </c>
       <c r="G10" s="7">
-        <v>825</v>
+        <v>0</v>
       </c>
       <c r="H10" s="7">
         <v>35</v>
       </c>
       <c r="I10" s="7">
         <f t="shared" si="0"/>
-        <v>790</v>
+        <v>-35</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>24</v>
@@ -13287,22 +13476,25 @@
       <c r="L10" s="7" t="s">
         <v>775</v>
       </c>
+      <c r="M10" s="7" t="s">
+        <v>797</v>
+      </c>
     </row>
     <row r="11" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>867</v>
+        <v>798</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>792</v>
+        <v>799</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>868</v>
+        <v>800</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="G11" s="7">
         <v>3780</v>
@@ -13315,7 +13507,7 @@
         <v>3745</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>24</v>
@@ -13332,13 +13524,13 @@
         <v>19</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>852</v>
+        <v>801</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>793</v>
+        <v>802</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>794</v>
+        <v>803</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>41</v>
@@ -13368,13 +13560,13 @@
         <v>19</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>795</v>
+        <v>804</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>796</v>
+        <v>805</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>874</v>
+        <v>806</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>28</v>
@@ -13390,7 +13582,7 @@
         <v>-30</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>24</v>
@@ -13404,13 +13596,13 @@
         <v>19</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>797</v>
+        <v>807</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>798</v>
+        <v>808</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>75</v>
@@ -13440,13 +13632,13 @@
         <v>19</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>800</v>
+        <v>810</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>801</v>
+        <v>811</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>125</v>
@@ -13476,13 +13668,13 @@
         <v>19</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>803</v>
+        <v>813</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>858</v>
+        <v>814</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>859</v>
+        <v>815</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>125</v>
@@ -13494,7 +13686,7 @@
         <v>35</v>
       </c>
       <c r="I16" s="5">
-        <f>G16-H16</f>
+        <f t="shared" si="0"/>
         <v>4485</v>
       </c>
       <c r="J16" s="5" t="s">
@@ -13515,13 +13707,13 @@
         <v>19</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>804</v>
+        <v>816</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>805</v>
+        <v>817</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>853</v>
+        <v>818</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>32</v>
@@ -13551,13 +13743,13 @@
         <v>19</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>806</v>
+        <v>819</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>807</v>
+        <v>820</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>808</v>
+        <v>821</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>45</v>
@@ -13587,13 +13779,13 @@
         <v>19</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>810</v>
+        <v>823</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>850</v>
+        <v>824</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>139</v>
@@ -13623,13 +13815,13 @@
         <v>19</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>811</v>
+        <v>825</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>812</v>
+        <v>826</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>854</v>
+        <v>827</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>79</v>
@@ -13659,13 +13851,13 @@
         <v>19</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>813</v>
+        <v>828</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>814</v>
+        <v>829</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>864</v>
+        <v>830</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>45</v>
@@ -13695,13 +13887,13 @@
         <v>19</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>815</v>
+        <v>831</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>816</v>
+        <v>832</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>817</v>
+        <v>833</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>79</v>
@@ -13717,7 +13909,7 @@
         <v>1350</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K22" s="7" t="s">
         <v>24</v>
@@ -13731,13 +13923,13 @@
         <v>19</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>875</v>
+        <v>834</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>818</v>
+        <v>835</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>819</v>
+        <v>836</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>38</v>
@@ -13753,7 +13945,7 @@
         <v>840</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>24</v>
@@ -13767,13 +13959,13 @@
         <v>19</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>820</v>
+        <v>837</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>821</v>
+        <v>838</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>869</v>
+        <v>839</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>162</v>
@@ -13789,7 +13981,7 @@
         <v>880</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K24" s="7" t="s">
         <v>24</v>
@@ -13803,13 +13995,13 @@
         <v>19</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>860</v>
+        <v>840</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>822</v>
+        <v>841</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>861</v>
+        <v>842</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>62</v>
@@ -13842,7 +14034,7 @@
         <v>691</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>823</v>
+        <v>843</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>693</v>
@@ -13878,13 +14070,13 @@
         <v>19</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>856</v>
+        <v>844</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>824</v>
+        <v>845</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>857</v>
+        <v>846</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>41</v>
@@ -13914,13 +14106,13 @@
         <v>19</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>825</v>
+        <v>847</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>826</v>
+        <v>848</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>865</v>
+        <v>849</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>162</v>
@@ -13950,13 +14142,13 @@
         <v>19</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>862</v>
+        <v>850</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>827</v>
+        <v>851</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>863</v>
+        <v>852</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>152</v>
@@ -13986,13 +14178,13 @@
         <v>19</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>828</v>
+        <v>853</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>829</v>
+        <v>854</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>830</v>
+        <v>855</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>162</v>
@@ -14022,13 +14214,13 @@
         <v>19</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>831</v>
+        <v>856</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>832</v>
+        <v>857</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>833</v>
+        <v>858</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>45</v>
@@ -14058,13 +14250,13 @@
         <v>19</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>834</v>
+        <v>859</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>835</v>
+        <v>860</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>162</v>
@@ -14092,18 +14284,18 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>873</v>
+        <v>862</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>836</v>
+        <v>863</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>837</v>
+        <v>864</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>129</v>
@@ -14119,7 +14311,7 @@
         <v>890</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K33" s="7" t="s">
         <v>24</v>
@@ -14128,31 +14320,31 @@
         <v>775</v>
       </c>
     </row>
-    <row r="34" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B34" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>838</v>
+        <v>865</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>839</v>
+        <v>866</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>840</v>
+        <v>867</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>162</v>
       </c>
       <c r="G34" s="5">
-        <v>760</v>
+        <v>30</v>
       </c>
       <c r="H34" s="5">
         <v>30</v>
       </c>
       <c r="I34" s="5">
         <f t="shared" si="0"/>
-        <v>730</v>
+        <v>0</v>
       </c>
       <c r="J34" s="5" t="s">
         <v>23</v>
@@ -14163,19 +14355,22 @@
       <c r="L34" s="5" t="s">
         <v>775</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="M34" s="5" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B35" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>876</v>
+        <v>869</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>841</v>
+        <v>870</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>877</v>
+        <v>871</v>
       </c>
       <c r="F35" s="8" t="s">
         <v>28</v>
@@ -14191,7 +14386,7 @@
         <v>1380</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K35" s="7" t="s">
         <v>24</v>
@@ -14200,18 +14395,18 @@
         <v>775</v>
       </c>
     </row>
-    <row r="36" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B36" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>842</v>
+        <v>872</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>843</v>
+        <v>873</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>79</v>
@@ -14227,7 +14422,7 @@
         <v>460</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>24</v>
@@ -14236,7 +14431,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="37" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>18</v>
       </c>
@@ -14244,10 +14439,10 @@
         <v>19</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>844</v>
+        <v>875</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>846</v>
+        <v>876</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>75</v>
@@ -14272,7 +14467,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="38" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>18</v>
       </c>
@@ -14280,10 +14475,10 @@
         <v>19</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>847</v>
+        <v>877</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>845</v>
+        <v>878</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>32</v>
@@ -14308,7 +14503,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="39" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>18</v>
       </c>
@@ -14316,10 +14511,10 @@
         <v>19</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>848</v>
+        <v>879</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>849</v>
+        <v>880</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>152</v>
@@ -14342,6 +14537,949 @@
       </c>
       <c r="L39" s="3" t="s">
         <v>775</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:P26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="44.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="75.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>882</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>883</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>884</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="3">
+        <v>920</v>
+      </c>
+      <c r="H3" s="3">
+        <v>30</v>
+      </c>
+      <c r="I3" s="3">
+        <f t="shared" ref="I3:I26" si="0">G3-H3</f>
+        <v>890</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>886</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>919</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="3">
+        <v>940</v>
+      </c>
+      <c r="H4" s="3">
+        <v>20</v>
+      </c>
+      <c r="I4" s="3">
+        <f t="shared" si="0"/>
+        <v>920</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>887</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>888</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>935</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="5">
+        <v>945</v>
+      </c>
+      <c r="H5" s="5">
+        <v>25</v>
+      </c>
+      <c r="I5" s="5">
+        <f t="shared" si="0"/>
+        <v>920</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>891</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>930</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="5">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5">
+        <v>25</v>
+      </c>
+      <c r="I6" s="5">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>892</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>893</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="5">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5">
+        <v>25</v>
+      </c>
+      <c r="I7" s="5">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>895</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>921</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="3">
+        <v>790</v>
+      </c>
+      <c r="H8" s="3">
+        <v>30</v>
+      </c>
+      <c r="I8" s="3">
+        <f t="shared" si="0"/>
+        <v>760</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>924</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>925</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G9" s="3">
+        <v>30</v>
+      </c>
+      <c r="H9" s="3">
+        <v>30</v>
+      </c>
+      <c r="I9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>885</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>896</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>897</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>927</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G10" s="5">
+        <v>485</v>
+      </c>
+      <c r="H10" s="5">
+        <v>25</v>
+      </c>
+      <c r="I10" s="5">
+        <f t="shared" si="0"/>
+        <v>460</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>898</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>899</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>932</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="G11" s="5">
+        <v>800</v>
+      </c>
+      <c r="H11" s="5">
+        <v>30</v>
+      </c>
+      <c r="I11" s="5">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>900</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="G12" s="5">
+        <v>490</v>
+      </c>
+      <c r="H12" s="5">
+        <v>30</v>
+      </c>
+      <c r="I12" s="5">
+        <f t="shared" si="0"/>
+        <v>460</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>937</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>901</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>938</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="7">
+        <v>0</v>
+      </c>
+      <c r="H13" s="7">
+        <v>25</v>
+      </c>
+      <c r="I13" s="7">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>902</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>903</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="G14" s="5">
+        <v>810</v>
+      </c>
+      <c r="H14" s="5">
+        <v>20</v>
+      </c>
+      <c r="I14" s="5">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>904</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>905</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5">
+        <v>25</v>
+      </c>
+      <c r="I15" s="5">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>906</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>907</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G16" s="5">
+        <v>815</v>
+      </c>
+      <c r="H16" s="5">
+        <v>25</v>
+      </c>
+      <c r="I16" s="5">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>929</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>908</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>928</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>909</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>910</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>911</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G18" s="7">
+        <v>1105</v>
+      </c>
+      <c r="H18" s="7">
+        <v>25</v>
+      </c>
+      <c r="I18" s="7">
+        <f t="shared" si="0"/>
+        <v>1080</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>912</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>913</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>926</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="G19" s="5">
+        <v>650</v>
+      </c>
+      <c r="H19" s="5">
+        <v>30</v>
+      </c>
+      <c r="I19" s="5">
+        <f t="shared" si="0"/>
+        <v>620</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>915</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>916</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G20" s="7">
+        <v>1120</v>
+      </c>
+      <c r="H20" s="7">
+        <v>30</v>
+      </c>
+      <c r="I20" s="7">
+        <f t="shared" si="0"/>
+        <v>1090</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>920</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="G21" s="3">
+        <v>30</v>
+      </c>
+      <c r="H21" s="3">
+        <v>30</v>
+      </c>
+      <c r="I21" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="7">
+        <v>2355</v>
+      </c>
+      <c r="H22" s="7">
+        <v>35</v>
+      </c>
+      <c r="I22" s="7">
+        <f t="shared" si="0"/>
+        <v>2320</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>917</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>918</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G23" s="7">
+        <v>7030</v>
+      </c>
+      <c r="H23" s="7">
+        <v>50</v>
+      </c>
+      <c r="I23" s="7">
+        <f t="shared" si="0"/>
+        <v>6980</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G24" s="7">
+        <v>30</v>
+      </c>
+      <c r="H24" s="7">
+        <v>30</v>
+      </c>
+      <c r="I24" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>922</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>923</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3">
+        <v>40</v>
+      </c>
+      <c r="I25" s="3">
+        <f t="shared" si="0"/>
+        <v>-40</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G26" s="3">
+        <v>4710</v>
+      </c>
+      <c r="H26" s="3">
+        <v>50</v>
+      </c>
+      <c r="I26" s="3">
+        <f t="shared" si="0"/>
+        <v>4660</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>885</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 16th Oct report
</commit_message>
<xml_diff>
--- a/data/Oct/Data_Oct.xlsx
+++ b/data/Oct/Data_Oct.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Oct\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\TextExtractorTool\data\Oct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7DB919-D2AE-43E3-A43C-315ECF0E566B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72BCFD92-0529-4373-B701-89F0D3F3AE38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5505" uniqueCount="1715">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5507" uniqueCount="1717">
   <si>
     <t>THU 5</t>
   </si>
@@ -5194,6 +5194,12 @@
   </si>
   <si>
     <t>Số 17, Đường Số 13, Phường Bình Hưng Hòa</t>
+  </si>
+  <si>
+    <t>kh ck shop 960k</t>
+  </si>
+  <si>
+    <t>kh ck shop 1965k</t>
   </si>
 </sst>
 </file>
@@ -15869,14 +15875,14 @@
         <v>199</v>
       </c>
       <c r="G14" s="5">
-        <v>1965</v>
+        <v>0</v>
       </c>
       <c r="H14" s="5">
         <v>35</v>
       </c>
       <c r="I14" s="5">
         <f t="shared" si="0"/>
-        <v>1930</v>
+        <v>-35</v>
       </c>
       <c r="J14" s="5" t="s">
         <v>23</v>
@@ -15887,6 +15893,9 @@
       <c r="L14" s="5" t="s">
         <v>1608</v>
       </c>
+      <c r="M14" s="5" t="s">
+        <v>1716</v>
+      </c>
     </row>
     <row r="15" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
@@ -16193,14 +16202,14 @@
         <v>162</v>
       </c>
       <c r="G23" s="5">
-        <v>960</v>
+        <v>0</v>
       </c>
       <c r="H23" s="5">
         <v>30</v>
       </c>
       <c r="I23" s="5">
         <f t="shared" si="0"/>
-        <v>930</v>
+        <v>-30</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>23</v>
@@ -16210,6 +16219,9 @@
       </c>
       <c r="L23" s="5" t="s">
         <v>1608</v>
+      </c>
+      <c r="M23" s="5" t="s">
+        <v>1715</v>
       </c>
     </row>
     <row r="24" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update 18th Oct 2026 report
</commit_message>
<xml_diff>
--- a/data/Oct/Data_Oct.xlsx
+++ b/data/Oct/Data_Oct.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Oct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7DB919-D2AE-43E3-A43C-315ECF0E566B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56EF54CE-8CB1-42E6-9AC6-B2F4B2AFAEDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-10" sheetId="6" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="14-10" sheetId="17" r:id="rId12"/>
     <sheet name="15-10" sheetId="18" r:id="rId13"/>
     <sheet name="16-10" sheetId="19" r:id="rId14"/>
+    <sheet name="17-10" sheetId="20" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5505" uniqueCount="1715">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5784" uniqueCount="1796">
   <si>
     <t>THU 5</t>
   </si>
@@ -4872,39 +4873,63 @@
     <t>NGAY 16-10</t>
   </si>
   <si>
+    <t>Chi Nguyen</t>
+  </si>
+  <si>
+    <t>312 Lô G cư xá Thanh Đa, p. Bình Quới</t>
+  </si>
+  <si>
+    <t>16-10-2026</t>
+  </si>
+  <si>
+    <t>Milly Đỗ</t>
+  </si>
+  <si>
+    <t>HD067453</t>
+  </si>
+  <si>
+    <t>14/144/10/7 phạm hùng, bình hưng</t>
+  </si>
+  <si>
     <t>AT 16-10</t>
   </si>
   <si>
-    <t>16-10-2026</t>
-  </si>
-  <si>
-    <t>Milly Đỗ</t>
-  </si>
-  <si>
-    <t>HD067453</t>
-  </si>
-  <si>
-    <t>14/144/10/7 phạm hùng, bình hưng</t>
+    <t>.Endny/ HOANG MEO</t>
   </si>
   <si>
     <t>HD067328</t>
   </si>
   <si>
+    <t>22, ĐƯỜNG TÂN THỚI NHẤT 1B, PHƯỜNG TÂN THỚI NHẤT</t>
+  </si>
+  <si>
     <t>Mai Lê</t>
   </si>
   <si>
     <t>HD067391</t>
   </si>
   <si>
+    <t>204/B12 Nguyễn văn hưởng, p thảo điền</t>
+  </si>
+  <si>
+    <t>Bảo Uyên</t>
+  </si>
+  <si>
     <t>HD067329</t>
   </si>
   <si>
+    <t>5606a vinhome grand park ( Đ. cầu vồng, Long Bình)</t>
+  </si>
+  <si>
     <t>Trân Helen</t>
   </si>
   <si>
     <t>HD067483</t>
   </si>
   <si>
+    <t>36/15 Yên Thế, Phường Tân Sơn Hoà, Phường Tân Bình</t>
+  </si>
+  <si>
     <t>HD067368</t>
   </si>
   <si>
@@ -4914,12 +4939,18 @@
     <t>HD067357</t>
   </si>
   <si>
+    <t>1079 tạ quang bửu phường bình đông</t>
+  </si>
+  <si>
     <t>Thanh Thảo Sumi</t>
   </si>
   <si>
     <t>HD067392</t>
   </si>
   <si>
+    <t>Căn 16.07 toà A2 chung cư Hoàng Anh River View, số 37 đường Nguyễn Văn Hưởng, phường An Khánh (phường cũ là Thảo Điền)</t>
+  </si>
+  <si>
     <t>HD067386</t>
   </si>
   <si>
@@ -4941,30 +4972,51 @@
     <t>HD067569</t>
   </si>
   <si>
+    <t>Block D1, Chung cư Hoàng Anh Gia Lai 3, Đường Nguyễn Hữu Thọ, xã Phước Kiển</t>
+  </si>
+  <si>
+    <t>Việt Trinh</t>
+  </si>
+  <si>
     <t>HD067371</t>
   </si>
   <si>
+    <t>Số 42, Đường Phùng Hưng Phường Chợ Lớn</t>
+  </si>
+  <si>
     <t>Hồng Nguyễn</t>
   </si>
   <si>
     <t>HD067451</t>
   </si>
   <si>
+    <t>621 Tân Kỳ Tân Quý, P. Bình Hưng Hòa</t>
+  </si>
+  <si>
     <t>HD067377</t>
   </si>
   <si>
+    <t>chung cư sunrise city view block B</t>
+  </si>
+  <si>
     <t>Thao Yumi</t>
   </si>
   <si>
     <t>HD067551</t>
   </si>
   <si>
+    <t>Số 17, Đường Số 13, Phường Bình Hưng Hòa</t>
+  </si>
+  <si>
     <t>HD067598</t>
   </si>
   <si>
     <t>HD067527</t>
   </si>
   <si>
+    <t>156 Trần Nhân Tôn, phường Vườn Lài (phường 2)</t>
+  </si>
+  <si>
     <t>Veriska Erica</t>
   </si>
   <si>
@@ -4980,9 +5032,15 @@
     <t>96 hoàng hoa thám</t>
   </si>
   <si>
+    <t>THI (KT Ng)</t>
+  </si>
+  <si>
     <t>HD067570</t>
   </si>
   <si>
+    <t>39 Nguyen thi Thap khu dan cu him lam phuong tan hung ( me in nail)</t>
+  </si>
+  <si>
     <t>Dinh Luong</t>
   </si>
   <si>
@@ -4998,6 +5056,9 @@
     <t>HD067567</t>
   </si>
   <si>
+    <t>Veronica Nhà Màu Vàng, 216/26, Nguyễn Văn Hưởng, Phường An Khánh</t>
+  </si>
+  <si>
     <t>Đinh Lily</t>
   </si>
   <si>
@@ -5013,6 +5074,12 @@
     <t>HD067447</t>
   </si>
   <si>
+    <t>The Opera Biệt thự Valora Ik6.33 đường số 11, Lk6-33 mới đúng ạ, đường số 11, Xã Bình Hưng</t>
+  </si>
+  <si>
+    <t>Tố Như</t>
+  </si>
+  <si>
     <t>HD067550</t>
   </si>
   <si>
@@ -5028,9 +5095,15 @@
     <t>31/3 ung văn khiêm thạnh mỹ tây</t>
   </si>
   <si>
+    <t>Ngọc Hiền</t>
+  </si>
+  <si>
     <t>HD067584</t>
   </si>
   <si>
+    <t>13c lê thánh tôn</t>
+  </si>
+  <si>
     <t>Nguyễn Ngọc Thiên Hương</t>
   </si>
   <si>
@@ -5043,12 +5116,27 @@
     <t>HD067599</t>
   </si>
   <si>
+    <t>38A đường 3158A phạm thế hiển phường bình đông(phuong 7) Đối diệncổng trường THPT nguyễn văn linh</t>
+  </si>
+  <si>
+    <t>Jessicaa</t>
+  </si>
+  <si>
     <t>HD067352</t>
   </si>
   <si>
+    <t>17A Cộng Hòa, Tân Sơn Nhất</t>
+  </si>
+  <si>
+    <t>Chế Vân</t>
+  </si>
+  <si>
     <t>HD067563</t>
   </si>
   <si>
+    <t>496/1/56 dương quảng hàm phường an nhơn</t>
+  </si>
+  <si>
     <t>HD067601</t>
   </si>
   <si>
@@ -5073,79 +5161,34 @@
     <t>HD067573</t>
   </si>
   <si>
+    <t>andu dang</t>
+  </si>
+  <si>
+    <t>24/5G, Ấp Đông Lân, Xã Bà Điểm</t>
+  </si>
+  <si>
     <t>phương uyên</t>
   </si>
   <si>
-    <t>204/B12 Nguyễn văn hưởng, p thảo điền</t>
-  </si>
-  <si>
-    <t>Chế Vân</t>
-  </si>
-  <si>
-    <t>496/1/56 dương quảng hàm phường an nhơn</t>
-  </si>
-  <si>
-    <t>.Endny/ HOANG MEO</t>
-  </si>
-  <si>
-    <t>22, ĐƯỜNG TÂN THỚI NHẤT 1B, PHƯỜNG TÂN THỚI NHẤT</t>
-  </si>
-  <si>
-    <t>andu dang</t>
-  </si>
-  <si>
-    <t>24/5G, Ấp Đông Lân, Xã Bà Điểm</t>
-  </si>
-  <si>
-    <t>Veronica Nhà Màu Vàng, 216/26, Nguyễn Văn Hưởng, Phường An Khánh</t>
-  </si>
-  <si>
-    <t>Căn 16.07 toà A2 chung cư Hoàng Anh River View, số 37 đường Nguyễn Văn Hưởng, phường An Khánh (phường cũ là Thảo Điền)</t>
-  </si>
-  <si>
-    <t>Chi Nguyen</t>
-  </si>
-  <si>
-    <t>312 Lô G cư xá Thanh Đa, p. Bình Quới</t>
-  </si>
-  <si>
-    <t>Jessicaa</t>
-  </si>
-  <si>
-    <t>17A Cộng Hòa, Tân Sơn Nhất</t>
-  </si>
-  <si>
-    <t>Việt Trinh</t>
-  </si>
-  <si>
-    <t>Số 42, Đường Phùng Hưng Phường Chợ Lớn</t>
-  </si>
-  <si>
-    <t>36/15 Yên Thế, Phường Tân Sơn Hoà, Phường Tân Bình</t>
-  </si>
-  <si>
-    <t>Ngọc Hiền</t>
-  </si>
-  <si>
-    <t>13c lê thánh tôn</t>
-  </si>
-  <si>
-    <t>156 Trần Nhân Tôn, phường Vườn Lài (phường 2)</t>
-  </si>
-  <si>
-    <t>THI (KT Ng)</t>
-  </si>
-  <si>
-    <t>39 Nguyen thi Thap khu dan cu him lam phuong tan hung ( me in nail)</t>
-  </si>
-  <si>
     <t>290 An Dương Vương phường 4 (phường Chợ Quán mới)</t>
   </si>
   <si>
-    <t>chung cư sunrise city view block B</t>
-  </si>
-  <si>
-    <t>Block D1, Chung cư Hoàng Anh Gia Lai 3, Đường Nguyễn Hữu Thọ, xã Phước Kiển</t>
+    <t>KHONGKWAN</t>
+  </si>
+  <si>
+    <t>Ngõ 72 đường 18B, phường Bình Hưng Hòa A</t>
+  </si>
+  <si>
+    <t>Nguyễn Minh Hải ( Bow)</t>
+  </si>
+  <si>
+    <t>17 Đường Số 13 Bình Hưng Hòa</t>
+  </si>
+  <si>
+    <t>Minea</t>
+  </si>
+  <si>
+    <t>363 Hùng Vương, Phường 9</t>
   </si>
   <si>
     <t>DaRaVin</t>
@@ -5154,46 +5197,247 @@
     <t>301 Phạm Ngũ Lão, Phường Phạm Ngũ Lão</t>
   </si>
   <si>
-    <t>Minea</t>
-  </si>
-  <si>
-    <t>363 Hùng Vương, Phường 9</t>
-  </si>
-  <si>
-    <t>Ngõ 72 đường 18B, phường Bình Hưng Hòa A</t>
-  </si>
-  <si>
-    <t>KHONGKWAN</t>
-  </si>
-  <si>
-    <t>Nguyễn Minh Hải ( Bow)</t>
-  </si>
-  <si>
-    <t>17 Đường Số 13 Bình Hưng Hòa</t>
-  </si>
-  <si>
-    <t>38A đường 3158A phạm thế hiển phường bình đông(phuong 7) Đối diệncổng trường THPT nguyễn văn linh</t>
-  </si>
-  <si>
-    <t>The Opera Biệt thự Valora Ik6.33 đường số 11, Lk6-33 mới đúng ạ, đường số 11, Xã Bình Hưng</t>
-  </si>
-  <si>
-    <t>1079 tạ quang bửu phường bình đông</t>
-  </si>
-  <si>
-    <t>Bảo Uyên</t>
-  </si>
-  <si>
-    <t>5606a vinhome grand park ( Đ. cầu vồng, Long Bình)</t>
-  </si>
-  <si>
-    <t>Tố Như</t>
-  </si>
-  <si>
-    <t>621 Tân Kỳ Tân Quý, P. Bình Hưng Hòa</t>
-  </si>
-  <si>
-    <t>Số 17, Đường Số 13, Phường Bình Hưng Hòa</t>
+    <t>NGAY 17-10</t>
+  </si>
+  <si>
+    <t>HD067851</t>
+  </si>
+  <si>
+    <t>103/14B Trần Quang Diệu P Nhiêu Lộc</t>
+  </si>
+  <si>
+    <t>17-10-2026</t>
+  </si>
+  <si>
+    <t>Vương Huệ</t>
+  </si>
+  <si>
+    <t>HD067681</t>
+  </si>
+  <si>
+    <t>HD067789</t>
+  </si>
+  <si>
+    <t>107 đường 4 khu tái định cư 680ha khu phố 11 linh xuân</t>
+  </si>
+  <si>
+    <t>HD067857</t>
+  </si>
+  <si>
+    <t>HD067779</t>
+  </si>
+  <si>
+    <t>HD067675</t>
+  </si>
+  <si>
+    <t>Jessie Beauty</t>
+  </si>
+  <si>
+    <t>HD067755</t>
+  </si>
+  <si>
+    <t>HD067637</t>
+  </si>
+  <si>
+    <t>(Anna Hanh )</t>
+  </si>
+  <si>
+    <t>HD067782</t>
+  </si>
+  <si>
+    <t>Thảo Đoàn</t>
+  </si>
+  <si>
+    <t>HD067832</t>
+  </si>
+  <si>
+    <t>HD067663</t>
+  </si>
+  <si>
+    <t>HD067735</t>
+  </si>
+  <si>
+    <t>Nhi Phan</t>
+  </si>
+  <si>
+    <t>HD067698</t>
+  </si>
+  <si>
+    <t>HD067687</t>
+  </si>
+  <si>
+    <t>HD067665</t>
+  </si>
+  <si>
+    <t>W2429</t>
+  </si>
+  <si>
+    <t>HD067615</t>
+  </si>
+  <si>
+    <t>Candy Kim</t>
+  </si>
+  <si>
+    <t>HD067682</t>
+  </si>
+  <si>
+    <t>HD067696</t>
+  </si>
+  <si>
+    <t>HD067791</t>
+  </si>
+  <si>
+    <t>HD067816</t>
+  </si>
+  <si>
+    <t>Linh Trần</t>
+  </si>
+  <si>
+    <t>HD067700</t>
+  </si>
+  <si>
+    <t>Lữ Nhung Lữ Nhung</t>
+  </si>
+  <si>
+    <t>HD067826</t>
+  </si>
+  <si>
+    <t>Thư</t>
+  </si>
+  <si>
+    <t>HD067829</t>
+  </si>
+  <si>
+    <t>76 trần đình xu</t>
+  </si>
+  <si>
+    <t>Bé Lan</t>
+  </si>
+  <si>
+    <t>HD067852</t>
+  </si>
+  <si>
+    <t>95 đường 59, P14</t>
+  </si>
+  <si>
+    <t>( Cẩm Giang) Kim Sarang</t>
+  </si>
+  <si>
+    <t>HD067864</t>
+  </si>
+  <si>
+    <t>417 Hậu Giang</t>
+  </si>
+  <si>
+    <t>Fangfang</t>
+  </si>
+  <si>
+    <t>W2488</t>
+  </si>
+  <si>
+    <t>HD067898</t>
+  </si>
+  <si>
+    <t>624 Lê Thị Riêng, Thới An</t>
+  </si>
+  <si>
+    <t>188 Nguyễn Văn Công, P.3</t>
+  </si>
+  <si>
+    <t>Soya Su</t>
+  </si>
+  <si>
+    <t>102 man thiện</t>
+  </si>
+  <si>
+    <t>31/23 đường làng tăng phú phường tăng nhơn phú a</t>
+  </si>
+  <si>
+    <t>22 TÂN THỚI NHẤT 1B, Phường Tân Thới Nhất</t>
+  </si>
+  <si>
+    <t>WIND XPRESS ( vận chuyển Việt -&gt; thái ) Số 68 . Tân thới hiệp 14</t>
+  </si>
+  <si>
+    <t>Vy</t>
+  </si>
+  <si>
+    <t>Số 6 hẻm 153 đường quốc lộ 13, phường 26</t>
+  </si>
+  <si>
+    <t>Hiếu Phan</t>
+  </si>
+  <si>
+    <t>BS10A vinhomes grand park phường long bình</t>
+  </si>
+  <si>
+    <t>Phong 1407 –Block B - Chung cư Opal Riverside, Đường Số 2, Phường Hiệp Bình</t>
+  </si>
+  <si>
+    <t>Nguyen Hoang Ngoc Anh</t>
+  </si>
+  <si>
+    <t>44/36 đông hưng thuận 6 phường tân hưng thuận</t>
+  </si>
+  <si>
+    <t>HD067697</t>
+  </si>
+  <si>
+    <t>132 Bến Vân Đồn phường 6</t>
+  </si>
+  <si>
+    <t>huyền nguyễn</t>
+  </si>
+  <si>
+    <t>243/44/12 tôn đản p15</t>
+  </si>
+  <si>
+    <t>80 đg số 3 tân kiếng</t>
+  </si>
+  <si>
+    <t>Như Lê</t>
+  </si>
+  <si>
+    <t>95/70/2 lê văn lương phường tân hưng</t>
+  </si>
+  <si>
+    <t>Thúy</t>
+  </si>
+  <si>
+    <t>Đặng Trinh ( phòng 103 )</t>
+  </si>
+  <si>
+    <t>406/35 Cộng Hòa, Phường 13</t>
+  </si>
+  <si>
+    <t>A75/6B/2 Bạch Đằng,Phường 2</t>
+  </si>
+  <si>
+    <t>Tuyết Nhi</t>
+  </si>
+  <si>
+    <t>28 Tân hương phường Phú Thọ Hòa</t>
+  </si>
+  <si>
+    <t>Ngọc GiÀu</t>
+  </si>
+  <si>
+    <t>207 trần văn kiểu phường bình phú</t>
+  </si>
+  <si>
+    <t>Lê Huyền Trang</t>
+  </si>
+  <si>
+    <t>61 Đặng Minh Trứ phường Bảy Hiền</t>
+  </si>
+  <si>
+    <t>1041 Hồng Bàng, P.Phú Lâm</t>
+  </si>
+  <si>
+    <t>đơn chuyển AT 17-10</t>
+  </si>
+  <si>
+    <t>AT 17-10</t>
   </si>
 </sst>
 </file>
@@ -15384,10 +15628,12 @@
   <dimension ref="A1:P48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="115.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -15458,10 +15704,10 @@
         <v>19</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1684</v>
+        <v>1607</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>1685</v>
+        <v>1608</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>75</v>
@@ -15483,7 +15729,7 @@
         <v>24</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>83</v>
@@ -15494,13 +15740,13 @@
         <v>19</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>121</v>
@@ -15516,13 +15762,13 @@
         <v>3805</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="M4" s="7" t="s">
         <v>94</v>
@@ -15533,13 +15779,13 @@
         <v>19</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1678</v>
+        <v>1614</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>1612</v>
+        <v>1615</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>1679</v>
+        <v>1616</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>79</v>
@@ -15561,7 +15807,7 @@
         <v>24</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -15569,13 +15815,13 @@
         <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>1613</v>
+        <v>1617</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>1614</v>
+        <v>1618</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>1675</v>
+        <v>1619</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>41</v>
@@ -15597,7 +15843,7 @@
         <v>24</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -15605,13 +15851,13 @@
         <v>19</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>1710</v>
+        <v>1620</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>1615</v>
+        <v>1621</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>1711</v>
+        <v>1622</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>139</v>
@@ -15627,13 +15873,13 @@
         <v>790</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -15641,13 +15887,13 @@
         <v>19</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>1616</v>
+        <v>1623</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>1617</v>
+        <v>1624</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>1690</v>
+        <v>1625</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>152</v>
@@ -15669,7 +15915,7 @@
         <v>24</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -15680,7 +15926,7 @@
         <v>417</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>1618</v>
+        <v>1626</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>419</v>
@@ -15705,7 +15951,7 @@
         <v>24</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -15713,13 +15959,13 @@
         <v>19</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>1619</v>
+        <v>1627</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>1620</v>
+        <v>1628</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>1709</v>
+        <v>1629</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>58</v>
@@ -15735,13 +15981,13 @@
         <v>920</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -15749,13 +15995,13 @@
         <v>19</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1621</v>
+        <v>1630</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>1622</v>
+        <v>1631</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>1683</v>
+        <v>1632</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>41</v>
@@ -15777,7 +16023,7 @@
         <v>24</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -15788,10 +16034,10 @@
         <v>837</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>1623</v>
+        <v>1633</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>1624</v>
+        <v>1634</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>162</v>
@@ -15813,7 +16059,7 @@
         <v>24</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -15821,13 +16067,13 @@
         <v>19</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>1625</v>
+        <v>1635</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>1626</v>
+        <v>1636</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>1627</v>
+        <v>1637</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>788</v>
@@ -15843,13 +16089,13 @@
         <v>1550</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -15857,13 +16103,13 @@
         <v>19</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>1628</v>
+        <v>1638</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>1629</v>
+        <v>1639</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>1698</v>
+        <v>1640</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>199</v>
@@ -15885,7 +16131,7 @@
         <v>24</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -15893,13 +16139,13 @@
         <v>19</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>1688</v>
+        <v>1641</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>1630</v>
+        <v>1642</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>1689</v>
+        <v>1643</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>22</v>
@@ -15921,7 +16167,7 @@
         <v>24</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -15929,13 +16175,13 @@
         <v>19</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>1631</v>
+        <v>1644</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>1632</v>
+        <v>1645</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>1713</v>
+        <v>1646</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
@@ -15951,13 +16197,13 @@
         <v>760</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="17" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -15968,10 +16214,10 @@
         <v>436</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>1633</v>
+        <v>1647</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>1697</v>
+        <v>1648</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>162</v>
@@ -15993,7 +16239,7 @@
         <v>24</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="18" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16001,13 +16247,13 @@
         <v>19</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>1634</v>
+        <v>1649</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>1635</v>
+        <v>1650</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>1714</v>
+        <v>1651</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>28</v>
@@ -16023,13 +16269,13 @@
         <v>1080</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="19" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16040,7 +16286,7 @@
         <v>1482</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>1636</v>
+        <v>1652</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>1467</v>
@@ -16065,7 +16311,7 @@
         <v>24</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="20" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16076,10 +16322,10 @@
         <v>208</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>1637</v>
+        <v>1653</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>1693</v>
+        <v>1654</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>294</v>
@@ -16101,7 +16347,7 @@
         <v>24</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="21" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16109,10 +16355,10 @@
         <v>19</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>1638</v>
+        <v>1655</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>1639</v>
+        <v>1656</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>1489</v>
@@ -16137,7 +16383,7 @@
         <v>24</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="22" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16145,13 +16391,13 @@
         <v>19</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>1640</v>
+        <v>1657</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>1641</v>
+        <v>1658</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>1642</v>
+        <v>1659</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>152</v>
@@ -16173,7 +16419,7 @@
         <v>24</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="23" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16181,13 +16427,13 @@
         <v>19</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>1694</v>
+        <v>1660</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>1643</v>
+        <v>1661</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>1695</v>
+        <v>1662</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>162</v>
@@ -16209,7 +16455,7 @@
         <v>24</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="24" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16217,13 +16463,13 @@
         <v>19</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>1644</v>
+        <v>1663</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>1645</v>
+        <v>1664</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>1646</v>
+        <v>1665</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>294</v>
@@ -16245,7 +16491,7 @@
         <v>24</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="25" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16253,26 +16499,26 @@
         <v>19</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>1647</v>
+        <v>1666</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>1648</v>
+        <v>1667</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>1682</v>
+        <v>1668</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>41</v>
       </c>
       <c r="G25" s="3">
-        <v>920</v>
+        <v>720</v>
       </c>
       <c r="H25" s="3">
         <v>30</v>
       </c>
       <c r="I25" s="3">
         <f t="shared" si="0"/>
-        <v>890</v>
+        <v>690</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>24</v>
@@ -16281,7 +16527,7 @@
         <v>24</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>355</v>
@@ -16292,13 +16538,13 @@
         <v>19</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>1649</v>
+        <v>1669</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>1650</v>
+        <v>1670</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>1651</v>
+        <v>1671</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>121</v>
@@ -16314,13 +16560,13 @@
         <v>870</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K26" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="27" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16328,13 +16574,13 @@
         <v>19</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>1652</v>
+        <v>1672</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>1653</v>
+        <v>1673</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>1708</v>
+        <v>1674</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>121</v>
@@ -16350,13 +16596,13 @@
         <v>-35</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K27" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="28" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16364,13 +16610,13 @@
         <v>19</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>1712</v>
+        <v>1675</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>1654</v>
+        <v>1676</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>1655</v>
+        <v>1677</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>28</v>
@@ -16386,13 +16632,13 @@
         <v>-30</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K28" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="29" spans="2:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16400,13 +16646,13 @@
         <v>19</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>1656</v>
+        <v>1678</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>1657</v>
+        <v>1679</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>1658</v>
+        <v>1680</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>75</v>
@@ -16428,7 +16674,7 @@
         <v>24</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="30" spans="2:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16436,13 +16682,13 @@
         <v>19</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>1691</v>
+        <v>1681</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>1659</v>
+        <v>1682</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>1692</v>
+        <v>1683</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>45</v>
@@ -16464,7 +16710,7 @@
         <v>24</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="31" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16472,13 +16718,13 @@
         <v>19</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>1660</v>
+        <v>1684</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>1661</v>
+        <v>1685</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>1662</v>
+        <v>1686</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>139</v>
@@ -16494,13 +16740,13 @@
         <v>430</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K31" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="32" spans="2:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16511,10 +16757,10 @@
         <v>1155</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>1663</v>
+        <v>1687</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>1707</v>
+        <v>1688</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>58</v>
@@ -16530,13 +16776,13 @@
         <v>140</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K32" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="M32" s="7" t="s">
         <v>83</v>
@@ -16547,13 +16793,13 @@
         <v>19</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>1686</v>
+        <v>1689</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>1664</v>
+        <v>1690</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>1687</v>
+        <v>1691</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>152</v>
@@ -16575,7 +16821,7 @@
         <v>24</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="34" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16583,13 +16829,13 @@
         <v>19</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>1676</v>
+        <v>1692</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>1665</v>
+        <v>1693</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>1677</v>
+        <v>1694</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>32</v>
@@ -16611,7 +16857,7 @@
         <v>24</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="M34" s="3" t="s">
         <v>83</v>
@@ -16625,7 +16871,7 @@
         <v>819</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>1666</v>
+        <v>1695</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>821</v>
@@ -16650,7 +16896,7 @@
         <v>24</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="36" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16658,13 +16904,13 @@
         <v>19</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>1667</v>
+        <v>1696</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>1668</v>
+        <v>1697</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>1669</v>
+        <v>1698</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>41</v>
@@ -16686,7 +16932,7 @@
         <v>24</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="37" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16694,13 +16940,13 @@
         <v>19</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>1670</v>
+        <v>1699</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>1671</v>
+        <v>1700</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>1672</v>
+        <v>1701</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>75</v>
@@ -16722,7 +16968,7 @@
         <v>24</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="38" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16730,13 +16976,13 @@
         <v>19</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>1647</v>
+        <v>1666</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>1673</v>
+        <v>1702</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>1682</v>
+        <v>1668</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>41</v>
@@ -16758,7 +17004,7 @@
         <v>24</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>355</v>
@@ -16772,10 +17018,10 @@
         <v>19</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>1680</v>
+        <v>1703</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>1681</v>
+        <v>1704</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>35</v>
@@ -16797,7 +17043,7 @@
         <v>24</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="40" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16827,13 +17073,13 @@
         <v>2100</v>
       </c>
       <c r="J40" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K40" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="41" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16863,13 +17109,13 @@
         <v>-35</v>
       </c>
       <c r="J41" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K41" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L41" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="42" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -16880,10 +17126,10 @@
         <v>19</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1674</v>
+        <v>1705</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>1696</v>
+        <v>1706</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>22</v>
@@ -16905,7 +17151,7 @@
         <v>24</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="43" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16916,10 +17162,10 @@
         <v>19</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>1704</v>
+        <v>1707</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>1703</v>
+        <v>1708</v>
       </c>
       <c r="F43" s="8" t="s">
         <v>28</v>
@@ -16935,13 +17181,13 @@
         <v>-35</v>
       </c>
       <c r="J43" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K43" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L43" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="44" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -16977,7 +17223,7 @@
         <v>24</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="45" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -16988,10 +17234,10 @@
         <v>19</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>1705</v>
+        <v>1709</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>1706</v>
+        <v>1710</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>28</v>
@@ -17007,13 +17253,13 @@
         <v>-35</v>
       </c>
       <c r="J45" s="7" t="s">
-        <v>1607</v>
+        <v>1613</v>
       </c>
       <c r="K45" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L45" s="7" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="46" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -17049,7 +17295,7 @@
         <v>24</v>
       </c>
       <c r="L46" s="3" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="47" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -17060,10 +17306,10 @@
         <v>19</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>1701</v>
+        <v>1711</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>1702</v>
+        <v>1712</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>22</v>
@@ -17085,7 +17331,7 @@
         <v>24</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="48" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -17096,10 +17342,10 @@
         <v>19</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>1699</v>
+        <v>1713</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>1700</v>
+        <v>1714</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>45</v>
@@ -17121,7 +17367,1253 @@
         <v>24</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>1608</v>
+        <v>1609</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+  <dimension ref="A1:P34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="71.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="36.42578125" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1715</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>1783</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>1716</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>1717</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3" s="5">
+        <v>855</v>
+      </c>
+      <c r="H3" s="5">
+        <v>25</v>
+      </c>
+      <c r="I3" s="5">
+        <f t="shared" ref="I3:I34" si="0">G3-H3</f>
+        <v>830</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1719</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>1720</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>1780</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="G4" s="5">
+        <v>920</v>
+      </c>
+      <c r="H4" s="5">
+        <v>30</v>
+      </c>
+      <c r="I4" s="5">
+        <f t="shared" si="0"/>
+        <v>890</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>1721</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>1722</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="3">
+        <v>860</v>
+      </c>
+      <c r="H5" s="3">
+        <v>30</v>
+      </c>
+      <c r="I5" s="3">
+        <f t="shared" si="0"/>
+        <v>830</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>1778</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>1723</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>1779</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="5">
+        <v>1035</v>
+      </c>
+      <c r="H6" s="5">
+        <v>25</v>
+      </c>
+      <c r="I6" s="5">
+        <f t="shared" si="0"/>
+        <v>1010</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>1724</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="3">
+        <v>955</v>
+      </c>
+      <c r="H7" s="3">
+        <v>25</v>
+      </c>
+      <c r="I7" s="3">
+        <f t="shared" si="0"/>
+        <v>930</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>1781</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>1725</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>1782</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="G8" s="5">
+        <v>960</v>
+      </c>
+      <c r="H8" s="5">
+        <v>30</v>
+      </c>
+      <c r="I8" s="5">
+        <f t="shared" si="0"/>
+        <v>930</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>1726</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>1776</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="G9" s="5">
+        <v>785</v>
+      </c>
+      <c r="H9" s="5">
+        <v>25</v>
+      </c>
+      <c r="I9" s="5">
+        <f t="shared" si="0"/>
+        <v>760</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>1784</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>1727</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>1785</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5">
+        <v>25</v>
+      </c>
+      <c r="I10" s="5">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>1728</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>1775</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G11" s="3">
+        <v>790</v>
+      </c>
+      <c r="H11" s="3">
+        <v>30</v>
+      </c>
+      <c r="I11" s="3">
+        <f t="shared" si="0"/>
+        <v>760</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>1760</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>1761</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>1762</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3">
+        <v>30</v>
+      </c>
+      <c r="I12" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>1729</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>1730</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>1763</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3">
+        <v>25</v>
+      </c>
+      <c r="I13" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>1731</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>1732</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>1793</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="7">
+        <v>955</v>
+      </c>
+      <c r="H14" s="7">
+        <v>25</v>
+      </c>
+      <c r="I14" s="7">
+        <f t="shared" si="0"/>
+        <v>930</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>1791</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>1733</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>1792</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="G15" s="7">
+        <v>945</v>
+      </c>
+      <c r="H15" s="7">
+        <v>25</v>
+      </c>
+      <c r="I15" s="7">
+        <f t="shared" si="0"/>
+        <v>920</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>1734</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>1045</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G16" s="3">
+        <v>1110</v>
+      </c>
+      <c r="H16" s="3">
+        <v>30</v>
+      </c>
+      <c r="I16" s="3">
+        <f t="shared" si="0"/>
+        <v>1080</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>1735</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>1736</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>1767</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3">
+        <v>30</v>
+      </c>
+      <c r="I17" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>1737</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="7">
+        <v>1750</v>
+      </c>
+      <c r="H18" s="7">
+        <v>30</v>
+      </c>
+      <c r="I18" s="7">
+        <f t="shared" si="0"/>
+        <v>1720</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>1769</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>1738</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>1770</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0</v>
+      </c>
+      <c r="H19" s="3">
+        <v>20</v>
+      </c>
+      <c r="I19" s="3">
+        <f t="shared" si="0"/>
+        <v>-20</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>1739</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>1740</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>1768</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3">
+        <v>30</v>
+      </c>
+      <c r="I20" s="3">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>1741</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>1766</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" s="3">
+        <v>820</v>
+      </c>
+      <c r="H21" s="3">
+        <v>30</v>
+      </c>
+      <c r="I21" s="3">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>1764</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>1743</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>1765</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G22" s="3">
+        <v>900</v>
+      </c>
+      <c r="H22" s="3">
+        <v>30</v>
+      </c>
+      <c r="I22" s="3">
+        <f t="shared" si="0"/>
+        <v>870</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>1789</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>1744</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>1790</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G23" s="7">
+        <v>855</v>
+      </c>
+      <c r="H23" s="7">
+        <v>25</v>
+      </c>
+      <c r="I23" s="7">
+        <f t="shared" si="0"/>
+        <v>830</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>1771</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>1745</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>1772</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G24" s="3">
+        <v>1110</v>
+      </c>
+      <c r="H24" s="3">
+        <v>30</v>
+      </c>
+      <c r="I24" s="3">
+        <f t="shared" si="0"/>
+        <v>1080</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>1746</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>1747</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>1777</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G25" s="5">
+        <v>785</v>
+      </c>
+      <c r="H25" s="5">
+        <v>25</v>
+      </c>
+      <c r="I25" s="5">
+        <f t="shared" si="0"/>
+        <v>760</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>1748</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>1749</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>1788</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="G26" s="7">
+        <v>645</v>
+      </c>
+      <c r="H26" s="7">
+        <v>25</v>
+      </c>
+      <c r="I26" s="7">
+        <f t="shared" si="0"/>
+        <v>620</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>1750</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>1751</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>1752</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G27" s="5">
+        <v>665</v>
+      </c>
+      <c r="H27" s="5">
+        <v>25</v>
+      </c>
+      <c r="I27" s="5">
+        <f t="shared" si="0"/>
+        <v>640</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>1753</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>1754</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>1755</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>25</v>
+      </c>
+      <c r="I28" s="3">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>1756</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>1757</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>1773</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G29" s="3">
+        <v>1090</v>
+      </c>
+      <c r="H29" s="3">
+        <v>30</v>
+      </c>
+      <c r="I29" s="3">
+        <f t="shared" si="0"/>
+        <v>1060</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>1787</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>1758</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G30" s="7">
+        <v>600</v>
+      </c>
+      <c r="H30" s="7">
+        <v>30</v>
+      </c>
+      <c r="I30" s="7">
+        <f t="shared" si="0"/>
+        <v>570</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K30" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L30" s="7" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G31" s="7">
+        <v>13880</v>
+      </c>
+      <c r="H31" s="7">
+        <v>80</v>
+      </c>
+      <c r="I31" s="7">
+        <f t="shared" si="0"/>
+        <v>13800</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>1759</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>1786</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="G32" s="5">
+        <v>960</v>
+      </c>
+      <c r="H32" s="5">
+        <v>30</v>
+      </c>
+      <c r="I32" s="5">
+        <f t="shared" si="0"/>
+        <v>930</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L32" s="5" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="33" spans="2:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>1681</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>1682</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>1683</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G33" s="11">
+        <v>955</v>
+      </c>
+      <c r="H33" s="11">
+        <v>25</v>
+      </c>
+      <c r="I33" s="11">
+        <f t="shared" si="0"/>
+        <v>930</v>
+      </c>
+      <c r="J33" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L33" s="11" t="s">
+        <v>1609</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="N33" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="O33" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="P33" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" spans="2:16" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>1641</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>1642</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>1643</v>
+      </c>
+      <c r="F34" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="G34" s="17">
+        <v>785</v>
+      </c>
+      <c r="H34" s="17">
+        <v>25</v>
+      </c>
+      <c r="I34" s="17">
+        <f t="shared" si="0"/>
+        <v>760</v>
+      </c>
+      <c r="J34" s="17" t="s">
+        <v>1795</v>
+      </c>
+      <c r="K34" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="17" t="s">
+        <v>1609</v>
+      </c>
+      <c r="M34" s="17" t="s">
+        <v>1794</v>
       </c>
     </row>
   </sheetData>

</xml_diff>